<commit_message>
Rehearsal data no longer names real prompts
The sample rows on the judge page carried two actual prompt titles and
one-line descriptions, four days before the prompts unlock. Neutral rows
now (B-0 / P-0 'Rehearsal prompt'); the Blob copy was overwritten the same
way.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KwvhkRFo1Un1Gzzkg5pg7
</commit_message>
<xml_diff>
--- a/pipeline/sample-responses.xlsx
+++ b/pipeline/sample-responses.xlsx
@@ -481,10 +481,10 @@
         <v>Build Track</v>
       </c>
       <c r="J2" t="str">
-        <v>B-2: Thermal Shipping Decision Engine</v>
+        <v>B-0: Rehearsal prompt</v>
       </c>
       <c r="L2" t="str">
-        <v>A tool that takes a Shopify order export and returns a thermal packing decision per order using the forecast for the transit window.</v>
+        <v>A rehearsal entry. Real submissions replace this row at 2:00 on the 19th.</v>
       </c>
       <c r="M2" t="str">
         <v>https://example.com/alpha-demo</v>
@@ -493,7 +493,7 @@
         <v>https://youtu.be/dQw4w9WgXcQ</v>
       </c>
       <c r="O2" t="str">
-        <v>Upload the sample CSV on the home screen, then open the Daily Pack List tab.</v>
+        <v>The first button on the home screen.</v>
       </c>
       <c r="P2" t="str">
         <v>https://github.com/example/alpha</v>
@@ -502,7 +502,7 @@
         <v>Yes</v>
       </c>
       <c r="R2" t="str">
-        <v>Use zip code 67202 for a hot-day example. No login needed.</v>
+        <v>No login needed.</v>
       </c>
     </row>
     <row r="3">
@@ -531,10 +531,10 @@
         <v>Pitch Track</v>
       </c>
       <c r="K3" t="str">
-        <v>P-2: Own the Off-Peak</v>
+        <v>P-0: Rehearsal prompt</v>
       </c>
       <c r="L3" t="str">
-        <v>A summer subscription box for corporate clients, priced and planned around slow-season capacity.</v>
+        <v>A rehearsal entry. Real submissions replace this row at 2:00 on the 19th.</v>
       </c>
       <c r="M3" t="str">
         <v>https://example.com/beta-pitch</v>
@@ -543,7 +543,7 @@
         <v>https://youtu.be/dQw4w9WgXcQ</v>
       </c>
       <c r="O3" t="str">
-        <v>Start at the pricing slider on the landing page, then scroll to the projections.</v>
+        <v>The first slide.</v>
       </c>
       <c r="Q3" t="str">
         <v>Yes</v>
@@ -575,10 +575,10 @@
         <v>Build Track</v>
       </c>
       <c r="J4" t="str">
-        <v>B-4: Build Wildcard</v>
+        <v>B-0: Rehearsal prompt</v>
       </c>
       <c r="L4" t="str">
-        <v>A kiosk app for the retail counter that logs which truffles a walk-in customer chose so the shop learns its bestsellers by weekday.</v>
+        <v>A rehearsal entry. Real submissions replace this row at 2:00 on the 19th.</v>
       </c>
       <c r="M4" t="str">
         <v>https://example.com/gamma</v>
@@ -587,13 +587,13 @@
         <v>https://youtu.be/dQw4w9WgXcQ</v>
       </c>
       <c r="O4" t="str">
-        <v>Tap Start Order and pick any three chocolates.</v>
+        <v>The first button on the home screen.</v>
       </c>
       <c r="Q4" t="str">
         <v>Yes</v>
       </c>
       <c r="R4" t="str">
-        <v>Works best on a tablet-sized window.</v>
+        <v>Works best in a laptop-sized window.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>